<commit_message>
Merge LinkedIn URLs and correct tenure years from LinkedIn CSV
Process data/Cornell_NCSU_LinkedIn_260718.csv (per-affiliation Cornell/NCSU rows,
one person repeated per stint) into the roster via data/update_tools/
process_linkedin.py, taking only the reliable fields:

- Fill 160 LinkedIn URLs (were blank) → 135/136 profiles now link to LinkedIn.
- Fill 14 blank start years + 18 blank end years from Cornell/NCSU tenure, adding
  ~14 alumni to the timeline.
- Transfer 13 accurate end years where the roster wrongly said "present"/blank
  (leaving departed alumni no longer shown as ongoing); then hand-correct three:
  Sara Miller → present, Sarah McMorrow → 2026, Mohamed El-Walid → 2026.
- Current positions left untouched — the CSV only knows Cornell/NCSU affiliations,
  so it can't speak to where alumni are now.

Regenerated js/people-data.js + js/profiles-data.js.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people-roster.xlsx
+++ b/data/people-roster.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="28800" windowHeight="16980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="28800" windowHeight="16860" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N168"/>
+  <dimension ref="A1:N167"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -643,7 +643,11 @@
         </is>
       </c>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/edward-buckler-b0749212</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Principal Investigator — Research Geneticist, USDA-ARS; Adjunct Professor of Plant Breeding &amp; Genetics, Cornell University</t>
@@ -703,7 +707,11 @@
         </is>
       </c>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/nonoy-bandillo-6b629630</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Assistant Professor, North Dakota State University</t>
@@ -749,7 +757,11 @@
       </c>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/larabrindisi</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -808,7 +820,11 @@
           <t>https://pjblab.faculty.ucdavis.edu/</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Associate Professor, Plant Sciences, University of California, Davis</t>
@@ -858,7 +874,11 @@
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/charles-chen-0211152b</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Assistant Professor of Bioinformatics, Oklahoma State University</t>
@@ -894,14 +914,16 @@
       <c r="C7" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D7" s="2" t="n">
+        <v>2016</v>
       </c>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/chen-shu-yun-a796b949</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Visiting Postdoctoral Scientist (former)</t>
@@ -937,7 +959,11 @@
       </c>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ecimen001</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Postdoc (former)</t>
@@ -983,14 +1009,16 @@
       <c r="C9" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D9" s="2" t="n">
+        <v>2023</v>
       </c>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/germanocneto</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1045,7 +1073,11 @@
           <t>https://umbrellagenetics.org</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>Managing Director, Umbrella Genetics LLC (former Postdoc, 2006–2010)</t>
@@ -1092,7 +1124,11 @@
         </is>
       </c>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/joe-gage-13bb5457</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Assistant Professor, Crop and Soil Sciences, NC State University</t>
@@ -1138,10 +1174,8 @@
       <c r="C12" s="3" t="n">
         <v>2001</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D12" s="2" t="n">
+        <v>2004</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -1149,7 +1183,11 @@
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sherry-flint-garcia</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Research Geneticist, USDA-ARS; Adjunct Professor, University of Missouri</t>
@@ -1185,10 +1223,8 @@
       <c r="C13" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D13" s="2" t="n">
+        <v>2018</v>
       </c>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="2" t="n"/>
@@ -1232,14 +1268,16 @@
       <c r="C14" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D14" s="2" t="n">
+        <v>2021</v>
       </c>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/anju-giri-b0838997</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Postdoctoral Associate</t>
@@ -1280,10 +1318,16 @@
       <c r="C15" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="2" t="n">
+        <v>2025</v>
+      </c>
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/gnanagnanapragasam-niranjani</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1324,7 +1368,11 @@
       </c>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/amit-gur-0054291a</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Researcher, Israeli Agricultural Research Organization (former Postdoc)</t>
@@ -1370,7 +1418,11 @@
       </c>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/carlos-harjes</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Molecular Geneticist, Bayer (former Postdoc)</t>
@@ -1408,7 +1460,11 @@
       </c>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1463,7 +1519,11 @@
         </is>
       </c>
       <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/matias-kirst-6899051b</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Professor, University of Florida</t>
@@ -1513,7 +1573,11 @@
         </is>
       </c>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/omry-koren-02696411</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1536,7 +1600,11 @@
       </c>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1598,7 +1666,11 @@
       </c>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/huihui-li-5057142a</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Visiting Scientist</t>
@@ -1652,7 +1724,11 @@
           <t>http://publish.illinois.edu/thelipkalab/</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/alex-lipka-45aa7a2b</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Assistant Professor of Biometry, Crop Sciences, University of Illinois at Urbana-Champaign</t>
@@ -1749,7 +1825,11 @@
           <t>http://plantgeneticslab.weebly.com/</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/fei-lu-1a07b864</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Professor, Institute of Genetics and Developmental Biology, Chinese Academy of Sciences</t>
@@ -1790,7 +1870,11 @@
       </c>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/katherine-mejia-guerra</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Postdoc (former)</t>
@@ -1830,7 +1914,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>postdoc</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -1843,7 +1927,11 @@
       </c>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/btmonier</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1897,7 +1985,11 @@
           <t>http://www.cultivatingdiversity.org/</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sean-myles-bb052555</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Associate Professor, Faculty of Agriculture, Dalhousie University</t>
@@ -1938,10 +2030,18 @@
       <c r="C30" s="5" t="n">
         <v>2023</v>
       </c>
-      <c r="D30" s="2" t="n"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/jonathan-ojeda-53b2712b5</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1994,7 +2094,11 @@
       </c>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Postdoc (former)</t>
@@ -2045,7 +2149,11 @@
       </c>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/gael-pressoir-0720697</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>Executive Director, Chibas Bioenergy; Vice Dean for Research, Quisqueya University (former Postdoc)</t>
@@ -2091,7 +2199,11 @@
       </c>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ramu-punna-a4102848</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>Genomic Selection Application Coordinator (former)</t>
@@ -2132,10 +2244,8 @@
       <c r="C34" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D34" s="2" t="n">
+        <v>2021</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -2143,7 +2253,11 @@
         </is>
       </c>
       <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/guillaume-ramstein-85680336</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -2202,7 +2316,11 @@
           <t>https://sites.google.com/a/uncg.edu/david-remington-home/</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/david-remington-21198078</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Associate Professor, UNC Greensboro</t>
@@ -2243,7 +2361,11 @@
       </c>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/eli-rodgers-melnick-0a12825</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Postdoctoral Associate (former)</t>
@@ -2290,7 +2412,11 @@
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/maria-cinta-romay-alvarez-142a1a50</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>Project Manager</t>
@@ -2345,7 +2471,11 @@
           <t>https://www.breedinginsight.org/</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/moira-sheehan-8723151b</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>Director, Breeding Insight (former Postdoctoral Associate)</t>
@@ -2386,7 +2516,11 @@
       </c>
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/dr-nisha-singh-48a7b914</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>Postdoc (former)</t>
@@ -2436,7 +2570,11 @@
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/song-baoxing-77301a60</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -2484,7 +2622,11 @@
       </c>
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -2539,7 +2681,11 @@
           <t>https://www.nwmissouri.edu/naturalsciences/directory/thornsberry.htm</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>Faculty, Northwest Missouri State University (former Postdoc)</t>
@@ -2584,7 +2730,11 @@
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>Professor, National Maize Improvement Center, China Agricultural University</t>
@@ -2679,7 +2829,11 @@
       </c>
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>Senior Expert, African Observatory for STI (former Postdoc)</t>
@@ -2723,7 +2877,11 @@
           <t>https://wallacelab.uga.edu</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/jason-wallace-a874b845</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>Associate Professor, University of Georgia</t>
@@ -2782,7 +2940,11 @@
           <t>http://bri.caas.cn/en/scientists/faculty/87624.htm</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>Visiting Scientist</t>
@@ -2839,7 +3001,11 @@
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/jacob-washburn-99013937</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>Postdoc / Research Geneticist, USDA-ARS</t>
@@ -2890,7 +3056,11 @@
       </c>
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>Visiting Postdoc</t>
@@ -2942,7 +3112,11 @@
         </is>
       </c>
       <c r="F50" s="2" t="n"/>
-      <c r="G50" s="2" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>Postdoctoral Associate (former)</t>
@@ -2996,7 +3170,11 @@
           <t>https://sites.google.com/site/quantitativegeneticsmaize/home</t>
         </is>
       </c>
-      <c r="G51" s="2" t="n"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>Professor, Iowa State University</t>
@@ -3044,7 +3222,11 @@
       </c>
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/jingjing-zhai-866031303</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -3085,7 +3267,11 @@
       </c>
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/dong-zhang-01</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3106,7 +3292,11 @@
       </c>
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="n"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>Postdoctoral Associate (former)</t>
@@ -3150,7 +3340,11 @@
           <t>http://zzlab.net/</t>
         </is>
       </c>
-      <c r="G55" s="2" t="n"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/zhiwu-zhang-14080223</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>Professor, Crop and Soil Sciences, Washington State University</t>
@@ -3196,7 +3390,11 @@
       </c>
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/taozuo</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>Bioinformatics Scientist, Monsanto (former Postdoc)</t>
@@ -3234,7 +3432,11 @@
       </c>
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/szu-ping-chen-40746319a</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3277,7 +3479,11 @@
       </c>
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="2" t="n"/>
-      <c r="G58" s="2" t="n"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/henry-dawson-2b16b3173</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3313,14 +3519,16 @@
       <c r="C59" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D59" s="2" t="n">
+        <v>2026</v>
       </c>
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="2" t="n"/>
-      <c r="G59" s="2" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/mohamed-el-walid</t>
+        </is>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3363,7 +3571,11 @@
       </c>
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/taylorferebee</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3414,7 +3626,11 @@
           <t>https://blogs.cornell.edu/gorelab</t>
         </is>
       </c>
-      <c r="G61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/michael-gore-9046a790</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>Associate Professor, Plant Breeding &amp; Genetics, Cornell University</t>
@@ -3462,7 +3678,11 @@
       </c>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="2" t="n"/>
-      <c r="G62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/charlesohale</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3503,7 +3723,11 @@
       </c>
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="2" t="n"/>
-      <c r="G63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/tiaho</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3524,7 +3748,11 @@
       </c>
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="2" t="n"/>
-      <c r="G64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sarah-jensen-1652b784</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3567,7 +3795,11 @@
       </c>
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="2" t="n"/>
-      <c r="G65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/merrittkhaiphoburch</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3604,7 +3836,11 @@
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/beatrice-konadu-62a350231</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3645,7 +3881,11 @@
       </c>
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/karl-kremling-70593715</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3686,7 +3926,11 @@
       </c>
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sara-larsson-3053a542</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3729,7 +3973,11 @@
       </c>
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/zongyanliu</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3772,7 +4020,11 @@
       </c>
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="2" t="n"/>
-      <c r="G70" s="2" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/evan-long-97952886</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3813,7 +4065,11 @@
       </c>
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="2" t="n"/>
-      <c r="G71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/japeiffe</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3829,14 +4085,16 @@
       <c r="C72" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D72" s="2" t="n">
+        <v>2022</v>
       </c>
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/evanrr</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3873,7 +4131,11 @@
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="2" t="n"/>
-      <c r="G73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/j-alberto-romero-navarro-51a038139</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -3904,14 +4166,16 @@
       <c r="C74" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D74" s="2" t="n">
+        <v>2022</v>
       </c>
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="2" t="n"/>
-      <c r="G74" s="2" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/travis-rooney-45226540</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -3953,7 +4217,11 @@
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3976,7 +4244,11 @@
       </c>
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="2" t="n"/>
-      <c r="G76" s="2" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/aimeejschulz</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>Graduate Student</t>
@@ -4021,7 +4293,11 @@
         </is>
       </c>
       <c r="F77" s="2" t="n"/>
-      <c r="G77" s="2" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/kelly-swarts-5a8787b3</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>Assistant Professor, Umeå Plant Science Center</t>
@@ -4058,7 +4334,11 @@
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="2" t="n"/>
-      <c r="G78" s="2" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/arcadeo</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -4109,7 +4389,11 @@
       </c>
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/larissa-wilson-49b0291</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -4140,14 +4424,16 @@
       <c r="C80" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D80" s="2" t="n">
+        <v>2024</v>
       </c>
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="2" t="n"/>
-      <c r="G80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/travis-wrightsman</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
           <t>Graduate Student (former)</t>
@@ -4190,11 +4476,19 @@
           <t>visiting</t>
         </is>
       </c>
-      <c r="C81" s="5" t="n"/>
-      <c r="D81" s="2" t="n"/>
+      <c r="C81" s="5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>2017</v>
+      </c>
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="2" t="n"/>
-      <c r="G81" s="2" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ijeoma-akaogu-a3a64339</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4215,7 +4509,11 @@
       </c>
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="2" t="n"/>
-      <c r="G82" s="2" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4270,7 +4568,11 @@
         </is>
       </c>
       <c r="F85" s="2" t="n"/>
-      <c r="G85" s="2" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>Visiting Scientist</t>
@@ -4307,7 +4609,11 @@
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="2" t="n"/>
-      <c r="G86" s="2" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4328,7 +4634,11 @@
       </c>
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="2" t="n"/>
-      <c r="G87" s="2" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4349,7 +4659,11 @@
       </c>
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="2" t="n"/>
-      <c r="G88" s="2" t="n"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4370,7 +4684,11 @@
       </c>
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="2" t="n"/>
-      <c r="G89" s="2" t="n"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/meng-h</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4391,7 +4709,11 @@
         </is>
       </c>
       <c r="F90" s="2" t="n"/>
-      <c r="G90" s="2" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4412,7 +4734,11 @@
       </c>
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="2" t="n"/>
-      <c r="G91" s="2" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
           <t>Visiting Graduate Student (former)</t>
@@ -4444,7 +4770,11 @@
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="2" t="n"/>
-      <c r="G92" s="2" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4461,7 +4791,11 @@
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="2" t="n"/>
-      <c r="G93" s="2" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4474,11 +4808,19 @@
           <t>visiting</t>
         </is>
       </c>
-      <c r="C94" s="5" t="n"/>
-      <c r="D94" s="2" t="n"/>
+      <c r="C94" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>2025</v>
+      </c>
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="2" t="n"/>
-      <c r="G94" s="2" t="n"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/vittorio-pipoli-25b467131</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4499,7 +4841,11 @@
         </is>
       </c>
       <c r="F95" s="2" t="n"/>
-      <c r="G95" s="2" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H95" t="inlineStr">
         <is>
           <t>Visiting Student (former)</t>
@@ -4540,7 +4886,11 @@
       </c>
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="2" t="n"/>
-      <c r="G96" s="2" t="n"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/carlos-alexandre-ribeiro-1002a638</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4553,11 +4903,19 @@
           <t>visiting</t>
         </is>
       </c>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="2" t="n"/>
+      <c r="C97" s="5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>2010</v>
+      </c>
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="2" t="n"/>
-      <c r="G97" s="2" t="n"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/abdoul-aziz-saidou-30ba385</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4578,7 +4936,11 @@
       </c>
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="2" t="n"/>
-      <c r="G98" s="2" t="n"/>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4595,7 +4957,11 @@
       <c r="D99" s="2" t="n"/>
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="2" t="n"/>
-      <c r="G99" s="2" t="n"/>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ram-kumar-sharma-7636845</t>
+        </is>
+      </c>
       <c r="H99" t="inlineStr">
         <is>
           <t>Visiting Scientist (former, 2010–2011)</t>
@@ -4640,7 +5006,11 @@
           <t>https://kazusa.or.jp</t>
         </is>
       </c>
-      <c r="G100" s="2" t="n"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H100" t="inlineStr">
         <is>
           <t>Visiting Scientist (former)</t>
@@ -4672,7 +5042,11 @@
       <c r="D101" s="2" t="n"/>
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="2" t="n"/>
-      <c r="G101" s="2" t="n"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4697,7 +5071,11 @@
         </is>
       </c>
       <c r="F102" s="2" t="n"/>
-      <c r="G102" s="2" t="n"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4722,7 +5100,11 @@
           <t>https://www.sinica.edu.tw/en</t>
         </is>
       </c>
-      <c r="G103" s="2" t="n"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H103" t="inlineStr">
         <is>
           <t>Visiting Scientist (former)</t>
@@ -4754,7 +5136,11 @@
       <c r="D104" s="2" t="n"/>
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="2" t="n"/>
-      <c r="G104" s="2" t="n"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H104" t="inlineStr">
         <is>
           <t>Visiting Scientist (former)</t>
@@ -4800,7 +5186,11 @@
       </c>
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="2" t="n"/>
-      <c r="G105" s="2" t="n"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4825,7 +5215,11 @@
         </is>
       </c>
       <c r="F106" s="2" t="n"/>
-      <c r="G106" s="2" t="n"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4846,7 +5240,11 @@
       </c>
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="2" t="n"/>
-      <c r="G107" s="2" t="n"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4863,7 +5261,11 @@
       <c r="D108" s="2" t="n"/>
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="2" t="n"/>
-      <c r="G108" s="2" t="n"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H108" t="inlineStr">
         <is>
           <t>Visiting Scientist</t>
@@ -4905,7 +5307,11 @@
       <c r="D109" s="2" t="n"/>
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="2" t="n"/>
-      <c r="G109" s="2" t="n"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4926,7 +5332,11 @@
       </c>
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="2" t="n"/>
-      <c r="G110" s="2" t="n"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4947,7 +5357,11 @@
       </c>
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="2" t="n"/>
-      <c r="G111" s="2" t="n"/>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H111" t="inlineStr">
         <is>
           <t>Visiting Graduate Student (former)</t>
@@ -4989,7 +5403,11 @@
         </is>
       </c>
       <c r="F112" s="2" t="n"/>
-      <c r="G112" s="2" t="n"/>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ana-berthel</t>
+        </is>
+      </c>
       <c r="H112" t="inlineStr">
         <is>
           <t>Programmer</t>
@@ -5025,10 +5443,8 @@
       <c r="C113" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D113" s="2" t="n">
+        <v>2026</v>
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
@@ -5036,7 +5452,11 @@
         </is>
       </c>
       <c r="F113" s="2" t="n"/>
-      <c r="G113" s="2" t="n"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sarah-jane-mcmorrow-537302207</t>
+        </is>
+      </c>
       <c r="H113" t="inlineStr">
         <is>
           <t>Programmer</t>
@@ -5083,7 +5503,11 @@
         </is>
       </c>
       <c r="F114" s="2" t="n"/>
-      <c r="G114" s="2" t="n"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/thuy-la-4a5a67ba</t>
+        </is>
+      </c>
       <c r="H114" t="inlineStr">
         <is>
           <t>Technician</t>
@@ -5130,7 +5554,11 @@
         </is>
       </c>
       <c r="F115" s="2" t="n"/>
-      <c r="G115" s="2" t="n"/>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sara-miller-03b53a19b</t>
+        </is>
+      </c>
       <c r="H115" t="inlineStr">
         <is>
           <t>Business Director</t>
@@ -5177,7 +5605,11 @@
         </is>
       </c>
       <c r="F116" s="2" t="n"/>
-      <c r="G116" s="2" t="n"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H116" t="inlineStr">
         <is>
           <t>Programmer</t>
@@ -5224,7 +5656,11 @@
         </is>
       </c>
       <c r="F117" s="2" t="n"/>
-      <c r="G117" s="2" t="n"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/nick-lepak-8321ab4a</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
           <t>Field Manager</t>
@@ -5271,7 +5707,11 @@
         </is>
       </c>
       <c r="F118" s="2" t="n"/>
-      <c r="G118" s="2" t="n"/>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/bethany-fallon-econopouly-322a16164</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr">
         <is>
           <t>International Applied Genomics Lead</t>
@@ -5316,7 +5756,11 @@
         </is>
       </c>
       <c r="F119" s="2" t="n"/>
-      <c r="G119" s="2" t="n"/>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/terry-casstevens-391a1a</t>
+        </is>
+      </c>
       <c r="H119" t="inlineStr">
         <is>
           <t>Bioinformatics (former)</t>
@@ -5363,7 +5807,11 @@
         </is>
       </c>
       <c r="F120" s="2" t="n"/>
-      <c r="G120" s="2" t="n"/>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/peter-bradbury-2236a714</t>
+        </is>
+      </c>
       <c r="H120" t="inlineStr">
         <is>
           <t>Computational Biologist, USDA-ARS</t>
@@ -5404,7 +5852,11 @@
       </c>
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="2" t="n"/>
-      <c r="G121" s="2" t="n"/>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H121" t="inlineStr">
         <is>
           <t>Genomic Selection Application Coordinator (former)</t>
@@ -5453,7 +5905,11 @@
           <t>https://www.elshiregroup.co.nz</t>
         </is>
       </c>
-      <c r="G122" s="2" t="n"/>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
           <t>Sequencing Technology Lead (former, 2007–2015)</t>
@@ -5489,7 +5945,11 @@
       </c>
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="2" t="n"/>
-      <c r="G123" s="2" t="n"/>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/dallas-kroon</t>
+        </is>
+      </c>
       <c r="H123" t="inlineStr">
         <is>
           <t>Software Developer (former)</t>
@@ -5525,7 +5985,11 @@
       </c>
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="2" t="n"/>
-      <c r="G124" s="2" t="n"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H124" t="inlineStr">
         <is>
           <t>Programmer (former)</t>
@@ -5567,7 +6031,11 @@
         </is>
       </c>
       <c r="F125" s="2" t="n"/>
-      <c r="G125" s="2" t="n"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>https://0</t>
+        </is>
+      </c>
       <c r="H125" t="inlineStr">
         <is>
           <t>Senior Scientist (former)</t>
@@ -5614,7 +6082,11 @@
         </is>
       </c>
       <c r="F126" s="2" t="n"/>
-      <c r="G126" s="2" t="n"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/lynn-johnson-1355aaa</t>
+        </is>
+      </c>
       <c r="H126" t="inlineStr">
         <is>
           <t>Programmer (former)</t>
@@ -5655,7 +6127,11 @@
       </c>
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="2" t="n"/>
-      <c r="G127" s="2" t="n"/>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/nicholas-kaczmar-04605412</t>
+        </is>
+      </c>
       <c r="H127" t="inlineStr">
         <is>
           <t>Field and Lab Assistant (former)</t>
@@ -5696,7 +6172,11 @@
       </c>
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="2" t="n"/>
-      <c r="G128" s="2" t="n"/>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/bradley-rauh-amplify-science</t>
+        </is>
+      </c>
       <c r="H128" t="inlineStr">
         <is>
           <t>Researcher (former)</t>
@@ -5737,7 +6217,11 @@
       </c>
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="2" t="n"/>
-      <c r="G129" s="2" t="n"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/janu-verma-b79b8823</t>
+        </is>
+      </c>
       <c r="H129" t="inlineStr">
         <is>
           <t>Quantitative Researcher (former)</t>
@@ -5778,7 +6262,11 @@
       </c>
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="2" t="n"/>
-      <c r="G130" s="2" t="n"/>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H130" t="inlineStr">
         <is>
           <t>IT Specialist, USDA (former Programmer)</t>
@@ -5819,7 +6307,11 @@
       </c>
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="2" t="n"/>
-      <c r="G131" s="2" t="n"/>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H131" t="inlineStr">
         <is>
           <t>Programmer (former)</t>
@@ -5856,7 +6348,11 @@
       <c r="D132" s="2" t="n"/>
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="2" t="n"/>
-      <c r="G132" s="2" t="n"/>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H132" t="inlineStr">
         <is>
           <t>Programmer</t>
@@ -5893,7 +6389,11 @@
       <c r="D133" s="2" t="n"/>
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="2" t="n"/>
-      <c r="G133" s="2" t="n"/>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H133" t="inlineStr">
         <is>
           <t>Technician (former)</t>
@@ -5929,14 +6429,16 @@
       <c r="C134" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
+      <c r="D134" s="2" t="n">
+        <v>2016</v>
       </c>
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="2" t="n"/>
-      <c r="G134" s="2" t="n"/>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H134" t="inlineStr">
         <is>
           <t>Field Technician (former)</t>
@@ -5969,11 +6471,19 @@
           <t>staff</t>
         </is>
       </c>
-      <c r="C135" s="5" t="n"/>
-      <c r="D135" s="2" t="n"/>
+      <c r="C135" s="5" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>2009</v>
+      </c>
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="2" t="n"/>
-      <c r="G135" s="2" t="n"/>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H135" t="inlineStr">
         <is>
           <t>Molecular Biology Technician (former)</t>
@@ -6009,7 +6519,11 @@
       </c>
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="2" t="n"/>
-      <c r="G136" s="2" t="n"/>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H136" t="inlineStr">
         <is>
           <t>Lab Technician (former)</t>
@@ -6045,7 +6559,11 @@
       </c>
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="2" t="n"/>
-      <c r="G137" s="2" t="n"/>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H137" t="inlineStr">
         <is>
           <t>Lab Administrator (former)</t>
@@ -6086,7 +6604,11 @@
       </c>
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="2" t="n"/>
-      <c r="G138" s="2" t="n"/>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H138" t="inlineStr">
         <is>
           <t>Lab Manager (former)</t>
@@ -6118,7 +6640,11 @@
       <c r="D139" s="2" t="n"/>
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="2" t="n"/>
-      <c r="G139" s="2" t="n"/>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H139" t="inlineStr">
         <is>
           <t>Administrative Assistant</t>
@@ -6155,7 +6681,11 @@
       <c r="D140" s="2" t="n"/>
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="2" t="n"/>
-      <c r="G140" s="2" t="n"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H140" t="inlineStr">
         <is>
           <t>Tripsacum Field Technician (former)</t>
@@ -6188,11 +6718,19 @@
           <t>staff</t>
         </is>
       </c>
-      <c r="C141" s="5" t="n"/>
-      <c r="D141" s="2" t="n"/>
+      <c r="C141" s="5" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D141" s="2" t="n">
+        <v>2010</v>
+      </c>
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="2" t="n"/>
-      <c r="G141" s="2" t="n"/>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H141" t="inlineStr">
         <is>
           <t>Administrative Assistant (former)</t>
@@ -6225,11 +6763,19 @@
           <t>staff</t>
         </is>
       </c>
-      <c r="C142" s="5" t="n"/>
-      <c r="D142" s="2" t="n"/>
+      <c r="C142" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>2024</v>
+      </c>
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="2" t="n"/>
-      <c r="G142" s="2" t="n"/>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H142" t="inlineStr">
         <is>
           <t>Lab Technician</t>
@@ -6270,7 +6816,11 @@
       </c>
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="2" t="n"/>
-      <c r="G143" s="2" t="n"/>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H143" t="inlineStr">
         <is>
           <t>Robotics Engineering Technician</t>
@@ -6303,11 +6853,19 @@
           <t>staff</t>
         </is>
       </c>
-      <c r="C144" s="5" t="n"/>
-      <c r="D144" s="2" t="n"/>
+      <c r="C144" s="5" t="n">
+        <v>2004</v>
+      </c>
+      <c r="D144" s="2" t="n">
+        <v>2009</v>
+      </c>
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="2" t="n"/>
-      <c r="G144" s="2" t="n"/>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H144" t="inlineStr">
         <is>
           <t>Lab Technician (former)</t>
@@ -6348,7 +6906,11 @@
       </c>
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="2" t="n"/>
-      <c r="G145" s="2" t="n"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6391,7 +6953,11 @@
       </c>
       <c r="E146" s="4" t="n"/>
       <c r="F146" s="2" t="n"/>
-      <c r="G146" s="2" t="n"/>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H146" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6428,7 +6994,11 @@
       <c r="D147" s="2" t="n"/>
       <c r="E147" s="4" t="n"/>
       <c r="F147" s="2" t="n"/>
-      <c r="G147" s="2" t="n"/>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6449,7 +7019,11 @@
       </c>
       <c r="E148" s="4" t="n"/>
       <c r="F148" s="2" t="n"/>
-      <c r="G148" s="2" t="n"/>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H148" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6486,7 +7060,11 @@
       <c r="D149" s="2" t="n"/>
       <c r="E149" s="4" t="n"/>
       <c r="F149" s="2" t="n"/>
-      <c r="G149" s="2" t="n"/>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H149" t="inlineStr">
         <is>
           <t>Undergraduate Researcher (former)</t>
@@ -6514,11 +7092,19 @@
           <t>undergrad</t>
         </is>
       </c>
-      <c r="C150" s="5" t="n"/>
-      <c r="D150" s="2" t="n"/>
+      <c r="C150" s="5" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D150" s="2" t="n">
+        <v>2019</v>
+      </c>
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="2" t="n"/>
-      <c r="G150" s="2" t="n"/>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H150" t="inlineStr">
         <is>
           <t>Undergraduate Programmer</t>
@@ -6555,7 +7141,11 @@
       <c r="D151" s="2" t="n"/>
       <c r="E151" s="4" t="n"/>
       <c r="F151" s="2" t="n"/>
-      <c r="G151" s="2" t="n"/>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr">
         <is>
           <t>Student Intern</t>
@@ -6588,11 +7178,19 @@
           <t>undergrad</t>
         </is>
       </c>
-      <c r="C152" s="5" t="n"/>
-      <c r="D152" s="2" t="n"/>
+      <c r="C152" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>2024</v>
+      </c>
       <c r="E152" s="4" t="n"/>
       <c r="F152" s="2" t="n"/>
-      <c r="G152" s="2" t="n"/>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H152" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6629,7 +7227,11 @@
       <c r="D153" s="2" t="n"/>
       <c r="E153" s="4" t="n"/>
       <c r="F153" s="2" t="n"/>
-      <c r="G153" s="2" t="n"/>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H153" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6666,7 +7268,11 @@
       <c r="D154" s="2" t="n"/>
       <c r="E154" s="4" t="n"/>
       <c r="F154" s="2" t="n"/>
-      <c r="G154" s="2" t="n"/>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H154" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6700,10 +7306,18 @@
         </is>
       </c>
       <c r="C155" s="5" t="n"/>
-      <c r="D155" s="2" t="n"/>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
       <c r="E155" s="4" t="n"/>
       <c r="F155" s="2" t="n"/>
-      <c r="G155" s="2" t="n"/>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H155" t="inlineStr">
         <is>
           <t>Student Intern</t>
@@ -6736,11 +7350,19 @@
           <t>undergrad</t>
         </is>
       </c>
-      <c r="C156" s="5" t="n"/>
-      <c r="D156" s="2" t="n"/>
+      <c r="C156" s="5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="D156" s="2" t="n">
+        <v>2007</v>
+      </c>
       <c r="E156" s="4" t="n"/>
       <c r="F156" s="2" t="n"/>
-      <c r="G156" s="2" t="n"/>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6753,11 +7375,19 @@
           <t>undergrad</t>
         </is>
       </c>
-      <c r="C157" s="5" t="n"/>
-      <c r="D157" s="2" t="n"/>
+      <c r="C157" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>2022</v>
+      </c>
       <c r="E157" s="4" t="n"/>
       <c r="F157" s="2" t="n"/>
-      <c r="G157" s="2" t="n"/>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H157" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6794,7 +7424,11 @@
       <c r="D158" s="2" t="n"/>
       <c r="E158" s="4" t="n"/>
       <c r="F158" s="2" t="n"/>
-      <c r="G158" s="2" t="n"/>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H158" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6827,6 +7461,11 @@
           <t>undergrad</t>
         </is>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H159" t="inlineStr">
         <is>
           <t>Bioinformatics Intern</t>
@@ -6859,6 +7498,11 @@
           <t>visiting</t>
         </is>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H160" t="inlineStr">
         <is>
           <t>Visiting Student (former)</t>
@@ -6883,7 +7527,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Beth Kraft Sant</t>
+          <t>Emily Yi</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -6891,26 +7535,42 @@
           <t>grad</t>
         </is>
       </c>
+      <c r="C161" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D161" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Graduate Student (former)</t>
+          <t>Undergraduate Researcher</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Non-thesis master's student with the group at North Carolina State University who pursued an MD at the Osteopathic Medical School at Virginia Tech.</t>
+          <t>Undergraduate student interested in computational and statistical techniques to solve biological problems, especially in response to changing climate; working on understanding pleiotropy in maize.</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>ety8@cornell.edu</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>beth-kraft-sant.jpg</t>
+          <t>emily-yi.jpg</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Emily Yi</t>
+          <t>Ben Fehr</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -6918,31 +7578,42 @@
           <t>grad</t>
         </is>
       </c>
+      <c r="C162" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D162" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Undergraduate Researcher</t>
+          <t>Graduate Student</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Undergraduate student interested in computational and statistical techniques to solve biological problems, especially in response to changing climate; working on understanding pleiotropy in maize.</t>
+          <t>Computational Biology graduate student interested in leveraging big data and machine learning for food system equity and sustainability, currently working on BAHD enzyme identification in maize.</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>ety8@cornell.edu</t>
+          <t>bf325@cornell.edu</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>emily-yi.jpg</t>
+          <t>ben-fehr.jpg</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Ben Fehr</t>
+          <t>Timothy Reeves</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6950,31 +7621,42 @@
           <t>grad</t>
         </is>
       </c>
+      <c r="C163" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D163" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Graduate Student</t>
+          <t>Undergraduate Researcher</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Computational Biology graduate student interested in leveraging big data and machine learning for food system equity and sustainability, currently working on BAHD enzyme identification in maize.</t>
+          <t>Junior pursuing a B.S. in Agricultural Sciences at Cornell, studying sustainable plant breeding with interests in machine learning and big data applications to environmental and genetic data.</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>bf325@cornell.edu</t>
+          <t>tjr239@cornell.edu</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>ben-fehr.jpg</t>
+          <t>timothy-reeves.jpg</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Timothy Reeves</t>
+          <t>Cindy Guan</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6982,6 +7664,11 @@
           <t>grad</t>
         </is>
       </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
+        </is>
+      </c>
       <c r="H164" t="inlineStr">
         <is>
           <t>Undergraduate Researcher</t>
@@ -6989,128 +7676,116 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Junior pursuing a B.S. in Agricultural Sciences at Cornell, studying sustainable plant breeding with interests in machine learning and big data applications to environmental and genetic data.</t>
+          <t>Sophomore pursuing a B.A. in Biological Sciences at Cornell, working on cassava genome assembly and evolutionary conservation using computational biology and statistics for sustainable global nutrition.</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>tjr239@cornell.edu</t>
+          <t>cg493@cornell.edu</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>timothy-reeves.jpg</t>
+          <t>cindy-guan.jpg</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Cindy Guan</t>
+          <t>Kristina Volkert</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>grad</t>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Undergraduate Researcher</t>
+          <t>Program Support Specialist (former)</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Sophomore pursuing a B.A. in Biological Sciences at Cornell, working on cassava genome assembly and evolutionary conservation using computational biology and statistics for sustainable global nutrition.</t>
+          <t>Served as the Program Support Specialist for the Buckler Lab and helped with travel, purchasing, visitors and website maintenance.</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>cg493@cornell.edu</t>
-        </is>
-      </c>
-      <c r="N165" t="inlineStr">
-        <is>
-          <t>cindy-guan.jpg</t>
+          <t>kmp279@cornell.edu</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Kristina Volkert</t>
+          <t>Jesse Zhou</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>grad</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Program Support Specialist (former)</t>
+          <t>Undergraduate Researcher</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Served as the Program Support Specialist for the Buckler Lab and helped with travel, purchasing, visitors and website maintenance.</t>
+          <t>Senior pursuing a B.S. in Plant Science at Cornell; researching soil's importance in crop growth models and assisting with maize field research in the Buckler Lab.</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>kmp279@cornell.edu</t>
+          <t>sz546@cornell.edu</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>jesse-zhou.jpg</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Jesse Zhou</t>
+          <t>Jennifer Heer</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>grad</t>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://#N/A</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Undergraduate Researcher</t>
+          <t>Research Technician (former)</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
-        <is>
-          <t>Senior pursuing a B.S. in Plant Science at Cornell; researching soil's importance in crop growth models and assisting with maize field research in the Buckler Lab.</t>
-        </is>
-      </c>
-      <c r="J167" t="inlineStr">
-        <is>
-          <t>sz546@cornell.edu</t>
-        </is>
-      </c>
-      <c r="N167" t="inlineStr">
-        <is>
-          <t>jesse-zhou.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Jennifer Heer</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>staff</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>Research Technician (former)</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
         <is>
           <t>Jennifer was a research technician with the group at North Carolina State University and worked on the Ra1 and the maize leafy homologues. She later went to work with TIGR.</t>
         </is>
@@ -7119,7 +7794,7 @@
   </sheetData>
   <autoFilter ref="A1:G158"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid role" error="Pick one of: pi, postdoc, grad, staff, undergrad, visiting" promptTitle="Role" prompt="Choose the person's role" type="list">
+    <dataValidation sqref="B2:B499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid role" error="Pick one of: pi, postdoc, grad, staff, undergrad, visiting" promptTitle="Role" prompt="Choose the person's role" type="list">
       <formula1>"pi,postdoc,grad,staff,undergrad,visiting"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Regenerate people data from further-completed roster
Another roster fill-in pass: timeline now places 151 people (was 148), with 139
current positions, 147 LinkedIn links, and 38 websites. 14 people still lack a
start year (profiles only, no timeline bar). Profiles unchanged at 136 (all bios;
kristina-volkert and jennifer-heer remain photoless).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people-roster.xlsx
+++ b/data/people-roster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/esb33/Developer/lab_site/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBFB15D-AEB9-C34B-8161-95018C455B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399F8A81-18AA-1A41-B614-55F6E061EA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,10 +60,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
           <t>4-digit year they left, or 'present' (blank = present)</t>
         </r>
@@ -102,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="949">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="1014">
   <si>
     <t>Name</t>
   </si>
@@ -1691,12 +1690,6 @@
     <t>Kenta Shirasawa</t>
   </si>
   <si>
-    <t>Senior Researcher, Kazusa DNA Research Institute</t>
-  </si>
-  <si>
-    <t>https://kazusa.or.jp</t>
-  </si>
-  <si>
     <t>Visiting Scientist (former)</t>
   </si>
   <si>
@@ -1706,15 +1699,9 @@
     <t>kenta-shirasawa.jpg</t>
   </si>
   <si>
-    <t>Mehraj Sofi</t>
-  </si>
-  <si>
     <t>Benjamin Stich</t>
   </si>
   <si>
-    <t>Professor, Heinrich Heine University Duesseldorf</t>
-  </si>
-  <si>
     <t>Mei-Hsiu Su</t>
   </si>
   <si>
@@ -1784,9 +1771,6 @@
     <t>Ana Berthel</t>
   </si>
   <si>
-    <t>Programmer, USDA-ARS</t>
-  </si>
-  <si>
     <t>https://linkedin.com/in/ana-berthel</t>
   </si>
   <si>
@@ -1805,9 +1789,6 @@
     <t>Sarah McMorrow</t>
   </si>
   <si>
-    <t>Bioinformatics, USDA-ARS</t>
-  </si>
-  <si>
     <t>https://linkedin.com/in/sarah-jane-mcmorrow-537302207</t>
   </si>
   <si>
@@ -1823,9 +1804,6 @@
     <t>Thuy La</t>
   </si>
   <si>
-    <t>Technician, USDA-ARS</t>
-  </si>
-  <si>
     <t>https://linkedin.com/in/thuy-la-4a5a67ba</t>
   </si>
   <si>
@@ -1916,9 +1894,6 @@
     <t>Terry Casstevens</t>
   </si>
   <si>
-    <t>Retired (formerly Bioinformatics Lead)</t>
-  </si>
-  <si>
     <t>https://linkedin.com/in/terry-casstevens-391a1a</t>
   </si>
   <si>
@@ -1985,9 +1960,6 @@
     <t>Dallas E. Kroon</t>
   </si>
   <si>
-    <t>https://linkedin.com/in/dallas-kroon</t>
-  </si>
-  <si>
     <t>Software Developer (former)</t>
   </si>
   <si>
@@ -2012,9 +1984,6 @@
     <t>Denise Costich</t>
   </si>
   <si>
-    <t>Retired (formerly CIMMYT Maize Germplasm Bank)</t>
-  </si>
-  <si>
     <t>Senior Scientist (former)</t>
   </si>
   <si>
@@ -2030,9 +1999,6 @@
     <t>Lynn Johnson</t>
   </si>
   <si>
-    <t>Statistical Consultant, Cornell University</t>
-  </si>
-  <si>
     <t>https://linkedin.com/in/lynn-johnson-1355aaa</t>
   </si>
   <si>
@@ -2051,9 +2017,6 @@
     <t>https://linkedin.com/in/nicholas-kaczmar-04605412</t>
   </si>
   <si>
-    <t>Field and Lab Assistant (former)</t>
-  </si>
-  <si>
     <t>Nick Kaczmar was a field and lab assistant in the Buckler Lab. He is now a Hydroponics/Aquaponics Specialist for the Horticulture Section of SIPS at Cornell University.</t>
   </si>
   <si>
@@ -2069,9 +2032,6 @@
     <t>https://linkedin.com/in/bradley-rauh-amplify-science</t>
   </si>
   <si>
-    <t>Researcher (former)</t>
-  </si>
-  <si>
     <t>Brad Rauh was a researcher with the group at North Carolina State University conducting a QTL experiment on nitrogen uptake in Arabidopsis and now serves as a Lab Technologist at Clemson University.</t>
   </si>
   <si>
@@ -2949,6 +2909,240 @@
   </si>
   <si>
     <t>Principal Researcher, Imaan Research, Niger</t>
+  </si>
+  <si>
+    <t>ramsharma@ihbt.res.in</t>
+  </si>
+  <si>
+    <t>http://www.ihbt.res.in/en/staff/scientific-staff?chronoform=sctdetail&amp;task=detail&amp;id=17</t>
+  </si>
+  <si>
+    <t>Chief Scientist, Professor, CSIR-IHBT, Palampur</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?user=sUto4QUAAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t>Laboratory Head, Kazusa DNA Research Institute</t>
+  </si>
+  <si>
+    <t>https://www.kazusa.or.jp/en-laboratories/en-advanced-department/en-plant-genome-lab/</t>
+  </si>
+  <si>
+    <t>Professor, SKUAST-Kashmir</t>
+  </si>
+  <si>
+    <t>mehrajpbg@skuastkashmir.ac.in</t>
+  </si>
+  <si>
+    <t>Mehrajuddin Sofi</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://scholar.google.com/citations%3Fuser%3Dx_PZgA4AAAAJ%26hl%3Den&amp;ved=2ahUKEwidjsr73t-VAxXbLFkFHZ--BzgQFnoECB0QAQ&amp;usg=AOvVaw3gc5gDncbrnG_Qe6dWeRwi</t>
+  </si>
+  <si>
+    <t>Head of Institute, Professor, Julius Kühn Institute</t>
+  </si>
+  <si>
+    <t>https://www.julius-kuehn.de/en/zl/staff/p/benjamin-stich</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://scholar.google.com/citations%3Fuser%3DHn20IkcAAAAJ%26hl%3Dde&amp;ved=2ahUKEwiBisXf_t-VAxXmjYkEHUX9BNEQFnoECA0QAQ&amp;usg=AOvVaw1XizLy5HWAD_o58Pa0Vedo</t>
+  </si>
+  <si>
+    <t>benjamin.stich@julius-kuehn.de</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/benjamin-stich-3544a563/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/mei-hsiu-su-97a853117/</t>
+  </si>
+  <si>
+    <t>Researcher, National Chung Hsing University</t>
+  </si>
+  <si>
+    <t>Professor, CIIDIR Unidad Sinaloa</t>
+  </si>
+  <si>
+    <t>Professor, Zhejiang University</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/profile/Qishan-Wang-7</t>
+  </si>
+  <si>
+    <t>wangqishan@zju.edu.cn</t>
+  </si>
+  <si>
+    <t>http://www.cas.zju.edu.cn/casenglish/15829/list.psp.</t>
+  </si>
+  <si>
+    <t>Research Leader, USDA-ARS, Pullman WA</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/marilyn-warburton-923b129/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://scholar.google.com/citations%3Fuser%3D5B9EX94AAAAJ%26hl%3Den&amp;ved=2ahUKEwjG3e78h-CVAxWCjokEHU4IFQ8QFnoECCcQAQ&amp;usg=AOvVaw3C-M8H3YV85BOJgsFFFw7Q</t>
+  </si>
+  <si>
+    <t>Business Director, BTI</t>
+  </si>
+  <si>
+    <t>Technician, Cornell</t>
+  </si>
+  <si>
+    <t>Programmer, BTU</t>
+  </si>
+  <si>
+    <t>Bioinformatics, Cornell</t>
+  </si>
+  <si>
+    <t>Bioinformatics Lead, USDA-ARS</t>
+  </si>
+  <si>
+    <t>https://sciprofiles.com/profile/2218909</t>
+  </si>
+  <si>
+    <t>Professor, Xinjiang Agricultural University</t>
+  </si>
+  <si>
+    <t>craie788@126.com &lt;craie788@126.com&gt;</t>
+  </si>
+  <si>
+    <t>Director &amp; Professor, Huazhong Agricultural University</t>
+  </si>
+  <si>
+    <t>yanfeiyan2004@163.com &lt;yanfeiyan2004@163.com&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Professor, Guangxi Academy of Agricultural Sciences，Nanning Guangxi </t>
+  </si>
+  <si>
+    <t>zhangl@cau.edu.cn</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/profile/Hongliang-Zhang-12</t>
+  </si>
+  <si>
+    <t>Professor, Sichuan Agricultural University</t>
+  </si>
+  <si>
+    <t>Project Manager, Computational Biologist</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/jeff-glaubitz-a794a6191/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://scholar.google.com/citations%3Fuser%3D2p550qoAAAAJ%26hl%3Den&amp;ved=2ahUKEwic6LPFueKVAxWbCnkGHcBBPeoQFnoECB4QAQ&amp;usg=AOvVaw1_XRPMJBEIIr6NbVGsYOb8</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://scholar.google.com/citations%3Fuser%3DGzS71NwAAAAJ%26hl%3Den&amp;ved=2ahUKEwjmzOCdvOKVAxUAlYkEHVvqFdcQFnoECBkQAQ&amp;usg=AOvVaw2KpM2scapSyx_wHLKTVLU5</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/dallas-kroon/</t>
+  </si>
+  <si>
+    <t>Scientist, International Food &amp; Fragrence</t>
+  </si>
+  <si>
+    <t>Retired (Bioinformatics Lead, Cornell)</t>
+  </si>
+  <si>
+    <t>Retired (Computational Biologist, USDA-ARS)</t>
+  </si>
+  <si>
+    <t>Retired (Programmer, Cornell University)</t>
+  </si>
+  <si>
+    <t>Principal Engineer, Everpure</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/yogesh-ramdoss-763448/</t>
+  </si>
+  <si>
+    <t>Retired (Director CIMMYT Maize Germplasm Bank)</t>
+  </si>
+  <si>
+    <t>Field Technician, USDA-ARS</t>
+  </si>
+  <si>
+    <t>Research Technician, USDA-ARS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principal Applied Scientist, Microsoft </t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/arturo-garcia-27872324/</t>
+  </si>
+  <si>
+    <t>IT Specialist, USDA-ARS</t>
+  </si>
+  <si>
+    <t>Teaching Lab Manager, Clemson University</t>
+  </si>
+  <si>
+    <t>Research Specialist, Cornell University</t>
+  </si>
+  <si>
+    <t>Informatics, Osthus GmbH, Aachen</t>
+  </si>
+  <si>
+    <t>Field Manager (former)</t>
+  </si>
+  <si>
+    <t>Software Engineer, IBM</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/natalie-stevens-4964b4162/</t>
+  </si>
+  <si>
+    <t>Slate Consultant</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/joshua-budka-7ba30562/</t>
+  </si>
+  <si>
+    <t>Head Grower, Gotham Greens</t>
+  </si>
+  <si>
+    <t>https://mattwie.se</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/sherry-whitt-3aaaa410a/</t>
+  </si>
+  <si>
+    <t>Global Manager Diagnostics, BASF</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/allison-krill-brown-110060314/</t>
+  </si>
+  <si>
+    <t>Strawberry Breeder, UC Davis</t>
+  </si>
+  <si>
+    <t>https://strawberry.ucdavis.edu/people/allison-krill-brown</t>
+  </si>
+  <si>
+    <t>Director, Chamblee OnStage</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/linda-rigamer-lirette-bba80732/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/elliot-richards-34b850119/</t>
+  </si>
+  <si>
+    <t>Graduate Student, Yale</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/patrick-o-briant/</t>
+  </si>
+  <si>
+    <t>Cultivation Station Farm Hub</t>
+  </si>
+  <si>
+    <t>Administrator, Cornell University</t>
   </si>
 </sst>
 </file>
@@ -3547,7 +3741,7 @@
         <v>2025</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>838</v>
+        <v>825</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
@@ -3592,7 +3786,7 @@
         <v>45</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>840</v>
+        <v>827</v>
       </c>
       <c r="H5" t="s">
         <v>47</v>
@@ -3657,7 +3851,7 @@
         <v>2016</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>841</v>
+        <v>828</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
@@ -3687,7 +3881,7 @@
         <v>2020</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>842</v>
+        <v>829</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
@@ -3726,7 +3920,7 @@
         <v>2023</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>843</v>
+        <v>830</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
@@ -3765,7 +3959,7 @@
         <v>2010</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>839</v>
+        <v>826</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>80</v>
@@ -3872,7 +4066,7 @@
         <v>2018</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>844</v>
+        <v>831</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
@@ -3905,7 +4099,7 @@
         <v>2021</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>845</v>
+        <v>832</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
@@ -3941,7 +4135,7 @@
         <v>2025</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>846</v>
+        <v>833</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
@@ -3974,10 +4168,10 @@
         <v>2007</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>847</v>
+        <v>834</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>848</v>
+        <v>835</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>120</v>
@@ -4012,7 +4206,7 @@
         <v>2007</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>849</v>
+        <v>836</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2" t="s">
@@ -4042,7 +4236,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>37</v>
+        <v>875</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
@@ -4081,7 +4275,7 @@
         <v>2004</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>850</v>
+        <v>837</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
@@ -4150,7 +4344,7 @@
         <v>2018</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>855</v>
+        <v>842</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -4169,7 +4363,7 @@
         <v>2009</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>851</v>
+        <v>838</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2" t="s">
@@ -4257,7 +4451,7 @@
         <v>167</v>
       </c>
       <c r="K24" t="s">
-        <v>852</v>
+        <v>839</v>
       </c>
       <c r="N24" t="s">
         <v>168</v>
@@ -4312,7 +4506,7 @@
         <v>2020</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>853</v>
+        <v>840</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
@@ -4351,7 +4545,7 @@
         <v>16</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>854</v>
+        <v>841</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2" t="s">
@@ -4424,7 +4618,9 @@
       <c r="D29" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>875</v>
+      </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2" t="s">
         <v>201</v>
@@ -4462,10 +4658,10 @@
         <v>2025</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>857</v>
+        <v>844</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>856</v>
+        <v>843</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>81</v>
@@ -4503,7 +4699,7 @@
         <v>2007</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>858</v>
+        <v>845</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2" t="s">
@@ -4539,7 +4735,7 @@
         <v>2018</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>859</v>
+        <v>846</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
@@ -4614,7 +4810,7 @@
         <v>2001</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>860</v>
+        <v>847</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>237</v>
@@ -4649,7 +4845,7 @@
         <v>2018</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>861</v>
+        <v>848</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2" t="s">
@@ -4682,10 +4878,10 @@
         <v>16</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>862</v>
+        <v>849</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>863</v>
+        <v>850</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>249</v>
@@ -4723,7 +4919,7 @@
         <v>2012</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>864</v>
+        <v>851</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>257</v>
@@ -4758,7 +4954,7 @@
         <v>2020</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>865</v>
+        <v>852</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2" t="s">
@@ -4794,7 +4990,7 @@
         <v>2022</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>866</v>
+        <v>853</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2" t="s">
@@ -4829,7 +5025,9 @@
       <c r="D40" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E40" s="4"/>
+      <c r="E40" s="4" t="s">
+        <v>875</v>
+      </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2" t="s">
         <v>81</v>
@@ -4867,13 +5065,13 @@
         <v>2003</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>868</v>
+        <v>855</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>282</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>867</v>
+        <v>854</v>
       </c>
       <c r="H41" t="s">
         <v>283</v>
@@ -4902,10 +5100,10 @@
         <v>2011</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>869</v>
+        <v>856</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>870</v>
+        <v>857</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>81</v>
@@ -4937,7 +5135,7 @@
         <v>2019</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>871</v>
+        <v>858</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2" t="s">
@@ -4973,11 +5171,11 @@
         <v>2006</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>873</v>
+        <v>860</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>872</v>
+        <v>859</v>
       </c>
       <c r="H44" t="s">
         <v>301</v>
@@ -5047,7 +5245,7 @@
         <v>288</v>
       </c>
       <c r="F46" t="s">
-        <v>874</v>
+        <v>861</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>81</v>
@@ -5124,10 +5322,10 @@
         <v>2021</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>875</v>
+        <v>862</v>
       </c>
       <c r="F48" t="s">
-        <v>876</v>
+        <v>863</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>81</v>
@@ -5142,7 +5340,7 @@
         <v>331</v>
       </c>
       <c r="K48" t="s">
-        <v>877</v>
+        <v>864</v>
       </c>
       <c r="L48" t="s">
         <v>332</v>
@@ -5168,7 +5366,7 @@
         <v>335</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>878</v>
+        <v>865</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>81</v>
@@ -5203,13 +5401,13 @@
         <v>2006</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>879</v>
+        <v>866</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>880</v>
+        <v>867</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>881</v>
+        <v>868</v>
       </c>
       <c r="H50" t="s">
         <v>341</v>
@@ -5241,7 +5439,7 @@
         <v>16</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>888</v>
+        <v>875</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2" t="s">
@@ -5274,7 +5472,7 @@
         <v>2014</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>884</v>
+        <v>871</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
@@ -5293,11 +5491,11 @@
         <v>2011</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>882</v>
+        <v>869</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
-        <v>883</v>
+        <v>870</v>
       </c>
       <c r="H53" t="s">
         <v>244</v>
@@ -5361,7 +5559,7 @@
         <v>2017</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>885</v>
+        <v>872</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2" t="s">
@@ -5457,7 +5655,7 @@
         <v>2026</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>886</v>
+        <v>873</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2" t="s">
@@ -5490,7 +5688,7 @@
         <v>2024</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>859</v>
+        <v>846</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2" t="s">
@@ -5523,7 +5721,7 @@
         <v>2009</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>887</v>
+        <v>874</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>392</v>
@@ -5592,7 +5790,7 @@
         <v>2017</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>889</v>
+        <v>876</v>
       </c>
       <c r="F62" s="2"/>
       <c r="G62" s="2" t="s">
@@ -5616,7 +5814,7 @@
         <v>2021</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>890</v>
+        <v>877</v>
       </c>
       <c r="F63" s="2"/>
       <c r="G63" s="2" t="s">
@@ -5649,7 +5847,7 @@
         <v>2024</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>891</v>
+        <v>878</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="2" t="s">
@@ -5715,7 +5913,7 @@
         <v>2018</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>892</v>
+        <v>879</v>
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2" t="s">
@@ -5748,7 +5946,7 @@
         <v>2013</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>893</v>
+        <v>880</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2" t="s">
@@ -5847,7 +6045,7 @@
         <v>2012</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>894</v>
+        <v>881</v>
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2" t="s">
@@ -5871,7 +6069,7 @@
         <v>2021</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>895</v>
+        <v>882</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2" t="s">
@@ -5904,7 +6102,7 @@
         <v>2016</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>896</v>
+        <v>883</v>
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2" t="s">
@@ -5934,7 +6132,7 @@
         <v>2022</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>897</v>
+        <v>884</v>
       </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2" t="s">
@@ -5958,7 +6156,7 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>898</v>
+        <v>885</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>370</v>
@@ -5970,10 +6168,10 @@
         <v>2001</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>900</v>
+        <v>887</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>899</v>
+        <v>886</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>81</v>
@@ -5993,7 +6191,7 @@
         <v>2024</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>901</v>
+        <v>888</v>
       </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2" t="s">
@@ -6026,7 +6224,7 @@
         <v>2016</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>902</v>
+        <v>889</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2" t="s">
@@ -6059,7 +6257,7 @@
         <v>2023</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>903</v>
+        <v>890</v>
       </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2" t="s">
@@ -6098,7 +6296,7 @@
         <v>2002</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>904</v>
+        <v>891</v>
       </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2" t="s">
@@ -6128,7 +6326,7 @@
         <v>2024</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>905</v>
+        <v>892</v>
       </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2" t="s">
@@ -6167,7 +6365,7 @@
         <v>2017</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>906</v>
+        <v>893</v>
       </c>
       <c r="F80" s="2"/>
       <c r="G80" s="2" t="s">
@@ -6188,10 +6386,10 @@
         <v>2014</v>
       </c>
       <c r="E81" t="s">
-        <v>913</v>
+        <v>900</v>
       </c>
       <c r="F81" t="s">
-        <v>914</v>
+        <v>901</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>81</v>
@@ -6202,7 +6400,7 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>907</v>
+        <v>894</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>489</v>
@@ -6214,11 +6412,11 @@
         <v>2023</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>908</v>
+        <v>895</v>
       </c>
       <c r="F82" s="2"/>
       <c r="G82" s="9" t="s">
-        <v>915</v>
+        <v>902</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.2">
@@ -6235,18 +6433,18 @@
         <v>2009</v>
       </c>
       <c r="E83" t="s">
-        <v>912</v>
+        <v>899</v>
       </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" t="s">
-        <v>911</v>
+        <v>898</v>
       </c>
       <c r="K83" t="s">
-        <v>910</v>
+        <v>897</v>
       </c>
       <c r="L83" t="s">
-        <v>909</v>
+        <v>896</v>
       </c>
     </row>
     <row r="84" spans="1:14" ht="28" x14ac:dyDescent="0.2">
@@ -6296,14 +6494,14 @@
         <v>2013</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>918</v>
+        <v>905</v>
       </c>
       <c r="F85" s="2"/>
       <c r="G85" s="2" t="s">
-        <v>917</v>
+        <v>904</v>
       </c>
       <c r="K85" t="s">
-        <v>916</v>
+        <v>903</v>
       </c>
     </row>
     <row r="86" spans="1:14" ht="28" x14ac:dyDescent="0.2">
@@ -6320,14 +6518,14 @@
         <v>2005</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>922</v>
+        <v>909</v>
       </c>
       <c r="F86" s="2"/>
       <c r="G86" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J86" t="s">
-        <v>923</v>
+        <v>910</v>
       </c>
     </row>
     <row r="87" spans="1:14" ht="28" x14ac:dyDescent="0.2">
@@ -6344,16 +6542,16 @@
         <v>2015</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>928</v>
+        <v>915</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>926</v>
+        <v>913</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>81</v>
       </c>
       <c r="K87" t="s">
-        <v>925</v>
+        <v>912</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
@@ -6370,16 +6568,16 @@
         <v>2014</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>927</v>
+        <v>914</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>933</v>
+        <v>920</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>502</v>
       </c>
       <c r="K88" t="s">
-        <v>932</v>
+        <v>919</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
@@ -6396,13 +6594,13 @@
         <v>2025</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>931</v>
+        <v>918</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>929</v>
+        <v>916</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>930</v>
+        <v>917</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="28" x14ac:dyDescent="0.2">
@@ -6419,10 +6617,10 @@
         <v>2011</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>936</v>
+        <v>923</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>934</v>
+        <v>921</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>81</v>
@@ -6434,10 +6632,10 @@
         <v>506</v>
       </c>
       <c r="J90" t="s">
-        <v>935</v>
+        <v>922</v>
       </c>
       <c r="K90" t="s">
-        <v>934</v>
+        <v>921</v>
       </c>
       <c r="N90" t="s">
         <v>507</v>
@@ -6445,7 +6643,7 @@
     </row>
     <row r="91" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>937</v>
+        <v>924</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>489</v>
@@ -6460,16 +6658,16 @@
         <v>494</v>
       </c>
       <c r="F91" t="s">
-        <v>939</v>
+        <v>926</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>81</v>
       </c>
       <c r="K91" t="s">
-        <v>795</v>
+        <v>782</v>
       </c>
       <c r="L91" t="s">
-        <v>938</v>
+        <v>925</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.2">
@@ -6486,16 +6684,16 @@
         <v>2014</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>941</v>
+        <v>928</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>940</v>
+        <v>927</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J92" s="10" t="s">
-        <v>942</v>
+        <v>929</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="18" x14ac:dyDescent="0.2">
@@ -6512,20 +6710,20 @@
         <v>2025</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>945</v>
+        <v>932</v>
       </c>
       <c r="F93" s="2"/>
       <c r="G93" s="2" t="s">
         <v>510</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>946</v>
+        <v>933</v>
       </c>
       <c r="K93" t="s">
-        <v>943</v>
+        <v>930</v>
       </c>
       <c r="L93" t="s">
-        <v>944</v>
+        <v>931</v>
       </c>
     </row>
     <row r="94" spans="1:14" ht="28" x14ac:dyDescent="0.2">
@@ -6546,7 +6744,7 @@
       </c>
       <c r="F94" s="2"/>
       <c r="G94" s="2" t="s">
-        <v>924</v>
+        <v>911</v>
       </c>
       <c r="H94" t="s">
         <v>513</v>
@@ -6575,7 +6773,7 @@
         <v>2015</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>947</v>
+        <v>934</v>
       </c>
       <c r="F95" s="2"/>
       <c r="G95" s="2" t="s">
@@ -6596,7 +6794,7 @@
         <v>2010</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>948</v>
+        <v>935</v>
       </c>
       <c r="F96" s="2"/>
       <c r="G96" s="2" t="s">
@@ -6617,16 +6815,16 @@
         <v>2007</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>921</v>
+        <v>908</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>920</v>
+        <v>907</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>81</v>
       </c>
       <c r="K97" t="s">
-        <v>919</v>
+        <v>906</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.2">
@@ -6636,10 +6834,18 @@
       <c r="B98" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C98" s="5"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="4"/>
-      <c r="F98" s="2"/>
+      <c r="C98" s="5">
+        <v>2010</v>
+      </c>
+      <c r="D98" s="2">
+        <v>2011</v>
+      </c>
+      <c r="E98" t="s">
+        <v>938</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>937</v>
+      </c>
       <c r="G98" s="2" t="s">
         <v>523</v>
       </c>
@@ -6648,6 +6854,9 @@
       </c>
       <c r="I98" t="s">
         <v>525</v>
+      </c>
+      <c r="J98" t="s">
+        <v>936</v>
       </c>
       <c r="K98" t="s">
         <v>526</v>
@@ -6663,145 +6872,190 @@
       <c r="B99" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C99" s="5"/>
-      <c r="D99" s="2"/>
+      <c r="C99" s="5">
+        <v>2013</v>
+      </c>
+      <c r="D99" s="2">
+        <v>2014</v>
+      </c>
       <c r="E99" s="4" t="s">
-        <v>529</v>
+        <v>940</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>530</v>
+        <v>941</v>
       </c>
       <c r="G99" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H99" t="s">
+        <v>529</v>
+      </c>
+      <c r="I99" t="s">
+        <v>530</v>
+      </c>
+      <c r="K99" t="s">
+        <v>939</v>
+      </c>
+      <c r="N99" t="s">
         <v>531</v>
-      </c>
-      <c r="I99" t="s">
-        <v>532</v>
-      </c>
-      <c r="N99" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>534</v>
+        <v>944</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C100" s="5"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="4"/>
+      <c r="C100" s="5">
+        <v>2015</v>
+      </c>
+      <c r="D100" s="2">
+        <v>2016</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>942</v>
+      </c>
       <c r="F100" s="2"/>
       <c r="G100" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="J100" s="10" t="s">
+        <v>943</v>
+      </c>
+      <c r="K100" t="s">
+        <v>945</v>
+      </c>
     </row>
     <row r="101" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>489</v>
       </c>
       <c r="C101" s="3">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="D101" s="3">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="F101" s="2"/>
+        <v>946</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>947</v>
+      </c>
       <c r="G101" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.2">
+        <v>950</v>
+      </c>
+      <c r="J101" t="s">
+        <v>949</v>
+      </c>
+      <c r="K101" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>489</v>
       </c>
       <c r="C102" s="3">
+        <v>2014</v>
+      </c>
+      <c r="D102" s="3">
         <v>2016</v>
       </c>
-      <c r="D102" s="3">
-        <v>2020</v>
-      </c>
-      <c r="E102" s="4"/>
+      <c r="E102" s="4" t="s">
+        <v>952</v>
+      </c>
       <c r="F102" s="2" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>81</v>
+        <v>951</v>
       </c>
       <c r="H102" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="I102" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="N102" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C103" s="5"/>
-      <c r="D103" s="2"/>
-      <c r="E103" s="4"/>
+      <c r="C103" s="5">
+        <v>2022</v>
+      </c>
+      <c r="D103" s="2">
+        <v>2023</v>
+      </c>
+      <c r="E103" s="4" t="s">
+        <v>953</v>
+      </c>
       <c r="F103" s="2"/>
       <c r="G103" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H103" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="I103" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="J103" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="L103" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="N103" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>489</v>
       </c>
       <c r="C104" s="3">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="D104" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E104" s="4"/>
-      <c r="F104" s="2"/>
+        <v>2011</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>954</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>957</v>
+      </c>
       <c r="G104" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="J104" t="s">
+        <v>956</v>
+      </c>
+      <c r="K104" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>489</v>
@@ -6810,19 +7064,22 @@
         <v>2005</v>
       </c>
       <c r="D105" s="3">
-        <v>2011</v>
+        <v>2005</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>320</v>
+        <v>958</v>
       </c>
       <c r="F105" s="2"/>
       <c r="G105" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.2">
+        <v>959</v>
+      </c>
+      <c r="K105" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>489</v>
@@ -6831,24 +7088,37 @@
         <v>2016</v>
       </c>
       <c r="D106" s="3">
-        <v>2018</v>
-      </c>
-      <c r="E106" s="4"/>
-      <c r="F106" s="2"/>
+        <v>2017</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>967</v>
+      </c>
+      <c r="F106" t="s">
+        <v>966</v>
+      </c>
       <c r="G106" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="J106" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C107" s="5"/>
-      <c r="D107" s="2"/>
-      <c r="E107" s="4"/>
+      <c r="C107" s="5">
+        <v>2018</v>
+      </c>
+      <c r="D107" s="2">
+        <v>2018</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>969</v>
+      </c>
       <c r="F107" s="2"/>
       <c r="G107" s="2" t="s">
         <v>81</v>
@@ -6857,55 +7127,71 @@
         <v>151</v>
       </c>
       <c r="I107" t="s">
+        <v>546</v>
+      </c>
+      <c r="J107" t="s">
+        <v>547</v>
+      </c>
+      <c r="L107" t="s">
+        <v>548</v>
+      </c>
+      <c r="N107" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" ht="42" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
         <v>550</v>
-      </c>
-      <c r="J107" t="s">
-        <v>551</v>
-      </c>
-      <c r="L107" t="s">
-        <v>552</v>
-      </c>
-      <c r="N107" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A108" s="2" t="s">
-        <v>554</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C108" s="5"/>
-      <c r="D108" s="2"/>
-      <c r="E108" s="4"/>
+      <c r="C108" s="5">
+        <v>2011</v>
+      </c>
+      <c r="D108" s="2">
+        <v>2011</v>
+      </c>
+      <c r="E108" s="4" t="s">
+        <v>971</v>
+      </c>
       <c r="F108" s="2"/>
       <c r="G108" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="J108" t="s">
+        <v>970</v>
+      </c>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A109" s="2" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>489</v>
       </c>
       <c r="C109" s="3">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="D109" s="3">
-        <v>2017</v>
-      </c>
-      <c r="E109" s="4"/>
-      <c r="F109" s="2"/>
+        <v>2013</v>
+      </c>
+      <c r="E109" t="s">
+        <v>288</v>
+      </c>
+      <c r="F109" t="s">
+        <v>973</v>
+      </c>
       <c r="G109" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="J109" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>489</v>
@@ -6914,9 +7200,11 @@
         <v>2013</v>
       </c>
       <c r="D110" s="3">
-        <v>2024</v>
-      </c>
-      <c r="E110" s="4"/>
+        <v>2013</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>974</v>
+      </c>
       <c r="F110" s="2"/>
       <c r="G110" s="2" t="s">
         <v>81</v>
@@ -6925,15 +7213,15 @@
         <v>505</v>
       </c>
       <c r="I110" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="N110" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>185</v>
@@ -6945,28 +7233,28 @@
         <v>16</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>560</v>
+        <v>963</v>
       </c>
       <c r="F111" s="2"/>
       <c r="G111" s="2" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="H111" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I111" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="J111" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="N111" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>185</v>
@@ -6978,127 +7266,127 @@
         <v>2026</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>567</v>
+        <v>964</v>
       </c>
       <c r="F112" s="2"/>
       <c r="G112" s="2" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="H112" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I112" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="J112" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="N112" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C113" s="3">
-        <v>2016</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>16</v>
+        <v>2019</v>
+      </c>
+      <c r="D113" s="2">
+        <v>2025</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>573</v>
+        <v>962</v>
       </c>
       <c r="F113" s="2"/>
       <c r="G113" s="2" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="H113" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="I113" t="s">
-        <v>576</v>
+        <v>569</v>
       </c>
       <c r="J113" t="s">
-        <v>577</v>
+        <v>570</v>
       </c>
       <c r="N113" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
-        <v>579</v>
+        <v>572</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C114" s="3">
-        <v>2014</v>
+        <v>2010</v>
       </c>
       <c r="D114" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>580</v>
+        <v>961</v>
       </c>
       <c r="F114" s="2"/>
       <c r="G114" s="2" t="s">
-        <v>581</v>
+        <v>574</v>
       </c>
       <c r="H114" t="s">
-        <v>580</v>
+        <v>573</v>
       </c>
       <c r="I114" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="J114" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="N114" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C115" s="3">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="D115" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>560</v>
+        <v>965</v>
       </c>
       <c r="F115" s="2"/>
       <c r="G115" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H115" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I115" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="J115" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="N115" t="s">
-        <v>588</v>
+        <v>581</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
-        <v>589</v>
+        <v>582</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>185</v>
@@ -7110,28 +7398,28 @@
         <v>16</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="F116" s="2"/>
       <c r="G116" s="2" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
       <c r="H116" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="I116" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="J116" t="s">
-        <v>594</v>
+        <v>587</v>
       </c>
       <c r="N116" t="s">
-        <v>595</v>
+        <v>588</v>
       </c>
     </row>
     <row r="117" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>185</v>
@@ -7143,28 +7431,28 @@
         <v>16</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
       <c r="F117" s="2"/>
       <c r="G117" s="2" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
       <c r="H117" t="s">
-        <v>599</v>
+        <v>592</v>
       </c>
       <c r="I117" t="s">
-        <v>600</v>
+        <v>593</v>
       </c>
       <c r="J117" t="s">
-        <v>601</v>
+        <v>594</v>
       </c>
       <c r="N117" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
     </row>
     <row r="118" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
-        <v>603</v>
+        <v>596</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>185</v>
@@ -7176,28 +7464,28 @@
         <v>2024</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>604</v>
+        <v>981</v>
       </c>
       <c r="F118" s="2"/>
       <c r="G118" s="2" t="s">
-        <v>605</v>
+        <v>597</v>
       </c>
       <c r="H118" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="I118" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="J118" t="s">
-        <v>608</v>
+        <v>600</v>
       </c>
       <c r="N118" t="s">
-        <v>609</v>
+        <v>601</v>
       </c>
     </row>
     <row r="119" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
-        <v>610</v>
+        <v>602</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>185</v>
@@ -7205,95 +7493,103 @@
       <c r="C119" s="3">
         <v>2003</v>
       </c>
-      <c r="D119" s="2" t="s">
-        <v>16</v>
+      <c r="D119" s="2">
+        <v>2024</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>611</v>
+        <v>982</v>
       </c>
       <c r="F119" s="2"/>
       <c r="G119" s="2" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="H119" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="I119" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="J119" t="s">
-        <v>614</v>
+        <v>606</v>
       </c>
       <c r="N119" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.2">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
-        <v>616</v>
+        <v>608</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C120" s="3">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="D120" s="3">
-        <v>2021</v>
-      </c>
-      <c r="E120" s="4"/>
+        <v>2016</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>975</v>
+      </c>
       <c r="F120" s="2"/>
       <c r="G120" s="2" t="s">
-        <v>81</v>
+        <v>976</v>
       </c>
       <c r="H120" t="s">
         <v>222</v>
       </c>
       <c r="I120" t="s">
-        <v>617</v>
+        <v>609</v>
       </c>
       <c r="J120" t="s">
-        <v>618</v>
+        <v>610</v>
+      </c>
+      <c r="K120" t="s">
+        <v>977</v>
       </c>
       <c r="N120" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C121" s="3">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="D121" s="3">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>622</v>
+        <v>614</v>
       </c>
       <c r="G121" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H121" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
       <c r="I121" t="s">
-        <v>624</v>
+        <v>616</v>
+      </c>
+      <c r="K121" t="s">
+        <v>978</v>
       </c>
       <c r="N121" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.2">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
-        <v>626</v>
+        <v>618</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>185</v>
@@ -7302,26 +7598,28 @@
         <v>2003</v>
       </c>
       <c r="D122" s="3">
-        <v>2010</v>
-      </c>
-      <c r="E122" s="4"/>
+        <v>2014</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>980</v>
+      </c>
       <c r="F122" s="2"/>
       <c r="G122" s="2" t="s">
-        <v>627</v>
+        <v>979</v>
       </c>
       <c r="H122" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="I122" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
       <c r="N122" t="s">
-        <v>630</v>
+        <v>621</v>
       </c>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A123" s="2" t="s">
-        <v>631</v>
+        <v>622</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>185</v>
@@ -7332,24 +7630,26 @@
       <c r="D123" s="3">
         <v>2007</v>
       </c>
-      <c r="E123" s="4"/>
+      <c r="E123" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="F123" s="2"/>
       <c r="G123" s="2" t="s">
-        <v>46</v>
+        <v>985</v>
       </c>
       <c r="H123" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
       <c r="I123" t="s">
-        <v>633</v>
+        <v>624</v>
       </c>
       <c r="N123" t="s">
-        <v>634</v>
+        <v>625</v>
       </c>
     </row>
     <row r="124" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
-        <v>635</v>
+        <v>626</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>185</v>
@@ -7357,32 +7657,32 @@
       <c r="C124" s="3">
         <v>2007</v>
       </c>
-      <c r="D124" s="2" t="s">
-        <v>16</v>
+      <c r="D124" s="2">
+        <v>2014</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>636</v>
+        <v>986</v>
       </c>
       <c r="F124" s="2"/>
       <c r="G124" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H124" t="s">
-        <v>637</v>
+        <v>627</v>
       </c>
       <c r="I124" t="s">
-        <v>638</v>
+        <v>628</v>
       </c>
       <c r="J124" t="s">
-        <v>639</v>
+        <v>629</v>
       </c>
       <c r="N124" t="s">
-        <v>640</v>
+        <v>630</v>
       </c>
     </row>
     <row r="125" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
-        <v>641</v>
+        <v>631</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>185</v>
@@ -7390,63 +7690,65 @@
       <c r="C125" s="3">
         <v>2014</v>
       </c>
-      <c r="D125" s="2" t="s">
-        <v>16</v>
+      <c r="D125" s="2">
+        <v>2025</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>642</v>
+        <v>983</v>
       </c>
       <c r="F125" s="2"/>
       <c r="G125" s="2" t="s">
-        <v>643</v>
+        <v>632</v>
       </c>
       <c r="H125" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
       <c r="I125" t="s">
-        <v>644</v>
+        <v>633</v>
       </c>
       <c r="J125" t="s">
-        <v>645</v>
+        <v>634</v>
       </c>
       <c r="N125" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.2">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14" ht="56" x14ac:dyDescent="0.2">
       <c r="A126" s="2" t="s">
-        <v>647</v>
+        <v>636</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C126" s="3">
-        <v>2017</v>
+        <v>2010</v>
       </c>
       <c r="D126" s="3">
-        <v>2024</v>
-      </c>
-      <c r="E126" s="4"/>
+        <v>2014</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>993</v>
+      </c>
       <c r="F126" s="2"/>
       <c r="G126" s="2" t="s">
-        <v>648</v>
-      </c>
-      <c r="H126" t="s">
-        <v>649</v>
+        <v>637</v>
+      </c>
+      <c r="H126" s="4" t="s">
+        <v>987</v>
       </c>
       <c r="I126" t="s">
-        <v>650</v>
+        <v>638</v>
       </c>
       <c r="J126" t="s">
-        <v>651</v>
+        <v>639</v>
       </c>
       <c r="N126" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.2">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14" ht="56" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
-        <v>653</v>
+        <v>641</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>185</v>
@@ -7455,29 +7757,31 @@
         <v>2000</v>
       </c>
       <c r="D127" s="3">
-        <v>2002</v>
-      </c>
-      <c r="E127" s="4"/>
+        <v>2003</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>992</v>
+      </c>
       <c r="F127" s="2"/>
       <c r="G127" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="H127" t="s">
-        <v>655</v>
+        <v>642</v>
+      </c>
+      <c r="H127" s="4" t="s">
+        <v>988</v>
       </c>
       <c r="I127" t="s">
-        <v>656</v>
+        <v>643</v>
       </c>
       <c r="J127" t="s">
-        <v>657</v>
+        <v>644</v>
       </c>
       <c r="N127" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.2">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14" ht="28" x14ac:dyDescent="0.2">
       <c r="A128" s="2" t="s">
-        <v>659</v>
+        <v>646</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>185</v>
@@ -7486,145 +7790,165 @@
         <v>2014</v>
       </c>
       <c r="D128" s="3">
-        <v>2017</v>
-      </c>
-      <c r="E128" s="4"/>
+        <v>2015</v>
+      </c>
+      <c r="E128" s="4" t="s">
+        <v>989</v>
+      </c>
       <c r="F128" s="2"/>
       <c r="G128" s="2" t="s">
-        <v>660</v>
+        <v>647</v>
       </c>
       <c r="H128" t="s">
-        <v>661</v>
+        <v>648</v>
       </c>
       <c r="I128" t="s">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="K128" t="s">
-        <v>663</v>
+        <v>650</v>
       </c>
       <c r="N128" t="s">
-        <v>664</v>
+        <v>651</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
-        <v>665</v>
+        <v>652</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C129" s="3">
-        <v>2007</v>
+        <v>2001</v>
       </c>
       <c r="D129" s="3">
-        <v>2020</v>
-      </c>
-      <c r="E129" s="4"/>
+        <v>2004</v>
+      </c>
+      <c r="E129" s="4" t="s">
+        <v>991</v>
+      </c>
       <c r="F129" s="2"/>
       <c r="G129" s="2" t="s">
-        <v>46</v>
+        <v>990</v>
       </c>
       <c r="H129" t="s">
-        <v>666</v>
+        <v>653</v>
       </c>
       <c r="I129" t="s">
-        <v>667</v>
+        <v>654</v>
       </c>
       <c r="J129" t="s">
-        <v>668</v>
+        <v>655</v>
       </c>
       <c r="N129" t="s">
-        <v>669</v>
+        <v>656</v>
       </c>
     </row>
     <row r="130" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
-        <v>670</v>
+        <v>657</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C130" s="3">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="D130" s="3">
-        <v>2015</v>
-      </c>
-      <c r="E130" s="4"/>
+        <v>2012</v>
+      </c>
+      <c r="E130" s="4" t="s">
+        <v>994</v>
+      </c>
       <c r="F130" s="2"/>
       <c r="G130" s="2" t="s">
         <v>46</v>
       </c>
       <c r="H130" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
       <c r="I130" t="s">
-        <v>671</v>
+        <v>658</v>
       </c>
       <c r="J130" t="s">
-        <v>672</v>
+        <v>659</v>
       </c>
       <c r="N130" t="s">
-        <v>673</v>
+        <v>660</v>
       </c>
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C131" s="5"/>
-      <c r="D131" s="2"/>
-      <c r="E131" s="4"/>
-      <c r="F131" s="2"/>
+      <c r="C131" s="5">
+        <v>2022</v>
+      </c>
+      <c r="D131" s="2">
+        <v>2023</v>
+      </c>
+      <c r="E131" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>1001</v>
+      </c>
       <c r="G131" s="2" t="s">
         <v>46</v>
       </c>
       <c r="H131" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I131" t="s">
-        <v>675</v>
+        <v>662</v>
       </c>
       <c r="J131" t="s">
-        <v>676</v>
+        <v>663</v>
       </c>
       <c r="N131" t="s">
-        <v>677</v>
+        <v>664</v>
       </c>
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A132" s="2" t="s">
-        <v>678</v>
+        <v>665</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C132" s="5"/>
-      <c r="D132" s="2"/>
-      <c r="E132" s="4"/>
+      <c r="C132" s="5">
+        <v>2020</v>
+      </c>
+      <c r="D132" s="2">
+        <v>2021</v>
+      </c>
+      <c r="E132" s="4" t="s">
+        <v>962</v>
+      </c>
       <c r="F132" s="2"/>
       <c r="G132" s="2" t="s">
         <v>46</v>
       </c>
       <c r="H132" t="s">
-        <v>679</v>
+        <v>666</v>
       </c>
       <c r="I132" t="s">
-        <v>680</v>
+        <v>667</v>
       </c>
       <c r="J132" t="s">
-        <v>681</v>
+        <v>668</v>
       </c>
       <c r="N132" t="s">
-        <v>682</v>
+        <v>669</v>
       </c>
     </row>
     <row r="133" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
-        <v>683</v>
+        <v>670</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>185</v>
@@ -7635,36 +7959,38 @@
       <c r="D133" s="2">
         <v>2016</v>
       </c>
-      <c r="E133" s="4"/>
+      <c r="E133" s="4" t="s">
+        <v>1000</v>
+      </c>
       <c r="F133" s="2"/>
       <c r="G133" s="2" t="s">
-        <v>46</v>
+        <v>999</v>
       </c>
       <c r="H133" t="s">
-        <v>684</v>
+        <v>671</v>
       </c>
       <c r="I133" t="s">
-        <v>685</v>
+        <v>672</v>
       </c>
       <c r="J133" t="s">
-        <v>686</v>
+        <v>673</v>
       </c>
       <c r="N133" t="s">
-        <v>687</v>
+        <v>674</v>
       </c>
     </row>
     <row r="134" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
-        <v>688</v>
+        <v>675</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C134" s="5">
-        <v>2008</v>
+        <v>2004</v>
       </c>
       <c r="D134" s="2">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="E134" s="4"/>
       <c r="F134" s="2"/>
@@ -7672,132 +7998,144 @@
         <v>46</v>
       </c>
       <c r="H134" t="s">
-        <v>689</v>
+        <v>676</v>
       </c>
       <c r="I134" t="s">
-        <v>690</v>
+        <v>677</v>
       </c>
       <c r="N134" t="s">
-        <v>691</v>
+        <v>678</v>
       </c>
     </row>
     <row r="135" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
-        <v>692</v>
+        <v>679</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C135" s="3">
-        <v>2003</v>
+        <v>2001</v>
       </c>
       <c r="D135" s="3">
-        <v>2005</v>
-      </c>
-      <c r="E135" s="4"/>
+        <v>2006</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>996</v>
+      </c>
       <c r="F135" s="2"/>
       <c r="G135" s="2" t="s">
         <v>46</v>
       </c>
       <c r="H135" t="s">
-        <v>693</v>
+        <v>995</v>
       </c>
       <c r="I135" t="s">
-        <v>694</v>
+        <v>681</v>
       </c>
       <c r="N135" t="s">
-        <v>695</v>
+        <v>682</v>
       </c>
     </row>
     <row r="136" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
-        <v>696</v>
+        <v>683</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C136" s="3">
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="D136" s="3">
-        <v>2009</v>
-      </c>
-      <c r="E136" s="4"/>
+        <v>2005</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>998</v>
+      </c>
       <c r="F136" s="2"/>
       <c r="G136" s="2" t="s">
-        <v>46</v>
+        <v>997</v>
       </c>
       <c r="H136" t="s">
-        <v>697</v>
+        <v>684</v>
       </c>
       <c r="I136" t="s">
-        <v>698</v>
+        <v>685</v>
       </c>
       <c r="J136" t="s">
-        <v>699</v>
+        <v>686</v>
       </c>
       <c r="N136" t="s">
-        <v>700</v>
+        <v>687</v>
       </c>
     </row>
     <row r="137" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
-        <v>701</v>
+        <v>688</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C137" s="3">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="D137" s="3">
-        <v>2006</v>
-      </c>
-      <c r="E137" s="4"/>
+        <v>2003</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>1003</v>
+      </c>
       <c r="F137" s="2"/>
       <c r="G137" s="2" t="s">
-        <v>46</v>
+        <v>1002</v>
       </c>
       <c r="H137" t="s">
-        <v>702</v>
+        <v>689</v>
       </c>
       <c r="I137" t="s">
-        <v>703</v>
+        <v>690</v>
       </c>
       <c r="N137" t="s">
-        <v>704</v>
+        <v>691</v>
       </c>
     </row>
     <row r="138" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
-        <v>705</v>
+        <v>692</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C138" s="5"/>
-      <c r="D138" s="2"/>
-      <c r="E138" s="4"/>
+      <c r="C138" s="5">
+        <v>2018</v>
+      </c>
+      <c r="D138" s="2">
+        <v>2022</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>1013</v>
+      </c>
       <c r="F138" s="2"/>
       <c r="G138" s="2" t="s">
         <v>46</v>
       </c>
       <c r="H138" t="s">
-        <v>706</v>
+        <v>693</v>
       </c>
       <c r="I138" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="J138" t="s">
-        <v>708</v>
+        <v>695</v>
       </c>
       <c r="N138" t="s">
-        <v>709</v>
+        <v>696</v>
       </c>
     </row>
     <row r="139" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
-        <v>710</v>
+        <v>697</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>185</v>
@@ -7810,21 +8148,21 @@
         <v>46</v>
       </c>
       <c r="H139" t="s">
-        <v>711</v>
+        <v>698</v>
       </c>
       <c r="I139" t="s">
-        <v>712</v>
+        <v>699</v>
       </c>
       <c r="J139" t="s">
-        <v>713</v>
+        <v>700</v>
       </c>
       <c r="N139" t="s">
-        <v>714</v>
+        <v>701</v>
       </c>
     </row>
     <row r="140" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
-        <v>715</v>
+        <v>702</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>185</v>
@@ -7835,27 +8173,29 @@
       <c r="D140" s="2">
         <v>2010</v>
       </c>
-      <c r="E140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>1007</v>
+      </c>
       <c r="F140" s="2"/>
       <c r="G140" s="2" t="s">
-        <v>46</v>
+        <v>1008</v>
       </c>
       <c r="H140" t="s">
-        <v>716</v>
+        <v>703</v>
       </c>
       <c r="I140" t="s">
-        <v>717</v>
+        <v>704</v>
       </c>
       <c r="J140" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="N140" t="s">
-        <v>719</v>
+        <v>706</v>
       </c>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
-        <v>720</v>
+        <v>707</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>185</v>
@@ -7866,58 +8206,62 @@
       <c r="D141" s="2">
         <v>2024</v>
       </c>
-      <c r="E141" s="4"/>
+      <c r="E141" s="4" t="s">
+        <v>1012</v>
+      </c>
       <c r="F141" s="2"/>
       <c r="G141" s="2" t="s">
-        <v>46</v>
+        <v>1011</v>
       </c>
       <c r="H141" t="s">
-        <v>721</v>
+        <v>708</v>
       </c>
       <c r="I141" t="s">
-        <v>722</v>
+        <v>709</v>
       </c>
       <c r="J141" t="s">
-        <v>723</v>
+        <v>710</v>
       </c>
       <c r="N141" t="s">
-        <v>724</v>
+        <v>711</v>
       </c>
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
-        <v>725</v>
+        <v>712</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C142" s="3">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="D142" s="3">
         <v>2019</v>
       </c>
-      <c r="E142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>1010</v>
+      </c>
       <c r="F142" s="2"/>
       <c r="G142" s="2" t="s">
-        <v>46</v>
+        <v>1009</v>
       </c>
       <c r="H142" t="s">
-        <v>726</v>
+        <v>713</v>
       </c>
       <c r="I142" t="s">
-        <v>727</v>
+        <v>714</v>
       </c>
       <c r="J142" t="s">
-        <v>728</v>
+        <v>715</v>
       </c>
       <c r="N142" t="s">
-        <v>729</v>
+        <v>716</v>
       </c>
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
-        <v>730</v>
+        <v>717</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>185</v>
@@ -7928,30 +8272,34 @@
       <c r="D143" s="2">
         <v>2009</v>
       </c>
-      <c r="E143" s="4"/>
-      <c r="F143" s="2"/>
+      <c r="E143" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>1006</v>
+      </c>
       <c r="G143" s="2" t="s">
-        <v>46</v>
+        <v>1004</v>
       </c>
       <c r="H143" t="s">
-        <v>693</v>
+        <v>680</v>
       </c>
       <c r="I143" t="s">
-        <v>731</v>
+        <v>718</v>
       </c>
       <c r="J143" t="s">
-        <v>732</v>
+        <v>719</v>
       </c>
       <c r="N143" t="s">
-        <v>733</v>
+        <v>720</v>
       </c>
     </row>
     <row r="144" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
-        <v>734</v>
+        <v>721</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C144" s="3">
         <v>2011</v>
@@ -7965,30 +8313,30 @@
         <v>46</v>
       </c>
       <c r="H144" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I144" t="s">
-        <v>737</v>
+        <v>724</v>
       </c>
       <c r="J144" t="s">
-        <v>738</v>
+        <v>725</v>
       </c>
       <c r="N144" t="s">
-        <v>739</v>
+        <v>726</v>
       </c>
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C145" s="3">
         <v>2023</v>
       </c>
-      <c r="D145" s="2" t="s">
-        <v>16</v>
+      <c r="D145" s="2">
+        <v>2025</v>
       </c>
       <c r="E145" s="4"/>
       <c r="F145" s="2"/>
@@ -7996,24 +8344,24 @@
         <v>46</v>
       </c>
       <c r="H145" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I145" t="s">
-        <v>741</v>
+        <v>728</v>
       </c>
       <c r="J145" t="s">
-        <v>742</v>
+        <v>729</v>
       </c>
       <c r="N145" t="s">
-        <v>743</v>
+        <v>730</v>
       </c>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
-        <v>744</v>
+        <v>731</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C146" s="5"/>
       <c r="D146" s="2"/>
@@ -8025,10 +8373,10 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
-        <v>745</v>
+        <v>732</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C147" s="3">
         <v>2019</v>
@@ -8042,24 +8390,24 @@
         <v>46</v>
       </c>
       <c r="H147" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I147" t="s">
-        <v>746</v>
+        <v>733</v>
       </c>
       <c r="J147" t="s">
-        <v>747</v>
+        <v>734</v>
       </c>
       <c r="N147" t="s">
-        <v>748</v>
+        <v>735</v>
       </c>
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
-        <v>749</v>
+        <v>736</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C148" s="5"/>
       <c r="D148" s="2"/>
@@ -8069,21 +8417,21 @@
         <v>46</v>
       </c>
       <c r="H148" t="s">
-        <v>750</v>
+        <v>737</v>
       </c>
       <c r="I148" t="s">
-        <v>751</v>
+        <v>738</v>
       </c>
       <c r="N148" t="s">
-        <v>752</v>
+        <v>739</v>
       </c>
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A149" s="2" t="s">
-        <v>753</v>
+        <v>740</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C149" s="5">
         <v>2018</v>
@@ -8097,24 +8445,24 @@
         <v>46</v>
       </c>
       <c r="H149" t="s">
-        <v>754</v>
+        <v>741</v>
       </c>
       <c r="I149" t="s">
-        <v>755</v>
+        <v>742</v>
       </c>
       <c r="J149" t="s">
-        <v>756</v>
+        <v>743</v>
       </c>
       <c r="N149" t="s">
-        <v>757</v>
+        <v>744</v>
       </c>
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
-        <v>758</v>
+        <v>745</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C150" s="5"/>
       <c r="D150" s="2"/>
@@ -8124,24 +8472,24 @@
         <v>46</v>
       </c>
       <c r="H150" t="s">
-        <v>759</v>
+        <v>746</v>
       </c>
       <c r="I150" t="s">
-        <v>760</v>
+        <v>747</v>
       </c>
       <c r="J150" t="s">
-        <v>761</v>
+        <v>748</v>
       </c>
       <c r="N150" t="s">
-        <v>762</v>
+        <v>749</v>
       </c>
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
-        <v>763</v>
+        <v>750</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C151" s="5">
         <v>2022</v>
@@ -8155,24 +8503,24 @@
         <v>46</v>
       </c>
       <c r="H151" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I151" t="s">
-        <v>764</v>
+        <v>751</v>
       </c>
       <c r="J151" t="s">
-        <v>765</v>
+        <v>752</v>
       </c>
       <c r="N151" t="s">
-        <v>766</v>
+        <v>753</v>
       </c>
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
-        <v>767</v>
+        <v>754</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C152" s="5"/>
       <c r="D152" s="2"/>
@@ -8182,24 +8530,24 @@
         <v>46</v>
       </c>
       <c r="H152" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I152" t="s">
-        <v>768</v>
+        <v>755</v>
       </c>
       <c r="J152" t="s">
-        <v>769</v>
+        <v>756</v>
       </c>
       <c r="N152" t="s">
-        <v>770</v>
+        <v>757</v>
       </c>
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
-        <v>771</v>
+        <v>758</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C153" s="5"/>
       <c r="D153" s="2"/>
@@ -8209,24 +8557,24 @@
         <v>46</v>
       </c>
       <c r="H153" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I153" t="s">
-        <v>772</v>
+        <v>759</v>
       </c>
       <c r="J153" t="s">
-        <v>773</v>
+        <v>760</v>
       </c>
       <c r="N153" t="s">
-        <v>774</v>
+        <v>761</v>
       </c>
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
-        <v>775</v>
+        <v>762</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C154" s="5"/>
       <c r="D154" s="2" t="s">
@@ -8238,24 +8586,24 @@
         <v>46</v>
       </c>
       <c r="H154" t="s">
-        <v>759</v>
+        <v>746</v>
       </c>
       <c r="I154" t="s">
-        <v>776</v>
+        <v>763</v>
       </c>
       <c r="J154" t="s">
-        <v>777</v>
+        <v>764</v>
       </c>
       <c r="N154" t="s">
-        <v>778</v>
+        <v>765</v>
       </c>
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
-        <v>779</v>
+        <v>766</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C155" s="5">
         <v>2006</v>
@@ -8271,10 +8619,10 @@
     </row>
     <row r="156" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
-        <v>780</v>
+        <v>767</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C156" s="5">
         <v>2022</v>
@@ -8288,24 +8636,24 @@
         <v>46</v>
       </c>
       <c r="H156" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I156" t="s">
-        <v>781</v>
+        <v>768</v>
       </c>
       <c r="J156" t="s">
-        <v>782</v>
+        <v>769</v>
       </c>
       <c r="N156" t="s">
-        <v>783</v>
+        <v>770</v>
       </c>
     </row>
     <row r="157" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
-        <v>784</v>
+        <v>771</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="C157" s="5"/>
       <c r="D157" s="2"/>
@@ -8315,44 +8663,44 @@
         <v>46</v>
       </c>
       <c r="H157" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I157" t="s">
-        <v>785</v>
+        <v>772</v>
       </c>
       <c r="J157" t="s">
-        <v>786</v>
+        <v>773</v>
       </c>
       <c r="N157" t="s">
-        <v>787</v>
+        <v>774</v>
       </c>
     </row>
     <row r="158" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>788</v>
+        <v>775</v>
       </c>
       <c r="B158" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="G158" t="s">
         <v>46</v>
       </c>
       <c r="H158" t="s">
-        <v>789</v>
+        <v>776</v>
       </c>
       <c r="I158" t="s">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="J158" t="s">
-        <v>791</v>
+        <v>778</v>
       </c>
       <c r="N158" t="s">
-        <v>792</v>
+        <v>779</v>
       </c>
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>793</v>
+        <v>780</v>
       </c>
       <c r="B159" t="s">
         <v>489</v>
@@ -8364,18 +8712,18 @@
         <v>513</v>
       </c>
       <c r="I159" t="s">
-        <v>794</v>
+        <v>781</v>
       </c>
       <c r="K159" t="s">
-        <v>795</v>
+        <v>782</v>
       </c>
       <c r="N159" t="s">
-        <v>796</v>
+        <v>783</v>
       </c>
     </row>
     <row r="160" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>797</v>
+        <v>784</v>
       </c>
       <c r="B160" t="s">
         <v>370</v>
@@ -8390,21 +8738,21 @@
         <v>46</v>
       </c>
       <c r="H160" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I160" t="s">
-        <v>798</v>
+        <v>785</v>
       </c>
       <c r="J160" t="s">
-        <v>799</v>
+        <v>786</v>
       </c>
       <c r="N160" t="s">
-        <v>800</v>
+        <v>787</v>
       </c>
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>801</v>
+        <v>788</v>
       </c>
       <c r="B161" t="s">
         <v>370</v>
@@ -8422,18 +8770,18 @@
         <v>372</v>
       </c>
       <c r="I161" t="s">
-        <v>802</v>
+        <v>789</v>
       </c>
       <c r="J161" t="s">
-        <v>803</v>
+        <v>790</v>
       </c>
       <c r="N161" t="s">
-        <v>804</v>
+        <v>791</v>
       </c>
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>805</v>
+        <v>792</v>
       </c>
       <c r="B162" t="s">
         <v>370</v>
@@ -8448,21 +8796,21 @@
         <v>46</v>
       </c>
       <c r="H162" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I162" t="s">
-        <v>806</v>
+        <v>793</v>
       </c>
       <c r="J162" t="s">
-        <v>807</v>
+        <v>794</v>
       </c>
       <c r="N162" t="s">
-        <v>808</v>
+        <v>795</v>
       </c>
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>809</v>
+        <v>796</v>
       </c>
       <c r="B163" t="s">
         <v>370</v>
@@ -8471,21 +8819,21 @@
         <v>46</v>
       </c>
       <c r="H163" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I163" t="s">
-        <v>810</v>
+        <v>797</v>
       </c>
       <c r="J163" t="s">
-        <v>811</v>
+        <v>798</v>
       </c>
       <c r="N163" t="s">
-        <v>812</v>
+        <v>799</v>
       </c>
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>813</v>
+        <v>800</v>
       </c>
       <c r="B164" t="s">
         <v>185</v>
@@ -8497,18 +8845,18 @@
         <v>46</v>
       </c>
       <c r="H164" t="s">
-        <v>814</v>
+        <v>801</v>
       </c>
       <c r="I164" t="s">
-        <v>815</v>
+        <v>802</v>
       </c>
       <c r="J164" t="s">
-        <v>816</v>
+        <v>803</v>
       </c>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>817</v>
+        <v>804</v>
       </c>
       <c r="B165" t="s">
         <v>370</v>
@@ -8517,21 +8865,21 @@
         <v>46</v>
       </c>
       <c r="H165" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="I165" t="s">
-        <v>818</v>
+        <v>805</v>
       </c>
       <c r="J165" t="s">
-        <v>819</v>
+        <v>806</v>
       </c>
       <c r="N165" t="s">
-        <v>820</v>
+        <v>807</v>
       </c>
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>821</v>
+        <v>808</v>
       </c>
       <c r="B166" t="s">
         <v>185</v>
@@ -8540,10 +8888,10 @@
         <v>46</v>
       </c>
       <c r="H166" t="s">
-        <v>822</v>
+        <v>809</v>
       </c>
       <c r="I166" t="s">
-        <v>823</v>
+        <v>810</v>
       </c>
     </row>
   </sheetData>
@@ -8558,9 +8906,11 @@
     <hyperlink ref="F49" r:id="rId2" xr:uid="{26A602FD-2CE8-254D-895C-C4961EA63DB4}"/>
     <hyperlink ref="G82" r:id="rId3" xr:uid="{F3B97894-51A3-B24A-8887-41297705C32D}"/>
     <hyperlink ref="J92" r:id="rId4" tooltip="r.paliwal@cgiar.org" display="mailto:r.paliwal@cgiar.org" xr:uid="{B366E188-1024-C143-BAE0-D3C32DD0895A}"/>
+    <hyperlink ref="J100" r:id="rId5" tooltip="mailto:Email%3Amehrajpbg@skuastkashmir.ac.in" display="mailto:Email%3Amehrajpbg@skuastkashmir.ac.in" xr:uid="{0DE9C552-7A29-4F40-A405-458CDBD4965A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <legacyDrawing r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -8574,7 +8924,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>824</v>
+        <v>811</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
@@ -8582,7 +8932,7 @@
     </row>
     <row r="3" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>825</v>
+        <v>812</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -8590,42 +8940,42 @@
     </row>
     <row r="5" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>826</v>
+        <v>813</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>827</v>
+        <v>814</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>828</v>
+        <v>815</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>829</v>
+        <v>816</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>830</v>
+        <v>817</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>831</v>
+        <v>818</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>832</v>
+        <v>819</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>833</v>
+        <v>820</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
@@ -8633,22 +8983,22 @@
     </row>
     <row r="14" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>834</v>
+        <v>821</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>835</v>
+        <v>822</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>836</v>
+        <v>823</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>